<commit_message>
Update VO_Manifest.xlsx with new data revisions
</commit_message>
<xml_diff>
--- a/HI02H04_L01_S01/VO_Manifest.xlsx
+++ b/HI02H04_L01_S01/VO_Manifest.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VO Manifest" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'VO Manifest'!$A$1:$B$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'VO Manifest'!$A$1:$B$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -470,456 +470,540 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>नमस्ते दोस्त! मैं हूँ स्विफ्टी। आइए, आज हम चित्र देखकर सही वाक्य मिलाना सीखें!</t>
+          <t>नमस्ते दोस्त! मैं हूँ स्विफ्टी! आज हम सीखेंगे—चित्रों को उनके सही वाक्यों से मिलाना।</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>vo_t1_narr</t>
+          <t>vo_tap_swiftee_replay</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>नमस्ते! आज हम सीखेंगे — तस्वीर के लिए सही वाक्य चुनना, और वाक्य के लिए सही तस्वीर चुनना। यह तस्वीर देखिए। इसके लिए सही वाक्य है — लड़का पेड़ के नीचे बैठा है। तस्वीर और वाक्य, दोनों एक जैसे हैं।</t>
+          <t>फिर से सुनने के लिए मुझ पर टैप करिए।</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>vo_t2_narr</t>
+          <t>vo_t1_instr</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>अब यह तस्वीर देखिए और वाक्य पढ़िए — लड़की साइकिल चला रही है। क्या यह वाक्य इस तस्वीर के लिए सही है? हाँ! तस्वीर में लड़की साइकिल चला रही है। हर शब्द को तस्वीर से मिलाकर देखिए — लड़की, साइकिल, चला रही है। सब सही हैं, इसलिए यह वाक्य सही है।</t>
+          <t>इस चित्र को ध्यान से देखिए और नीचे दिए गए वाक्य को पढ़िए।</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>vo_t3_narr</t>
+          <t>vo_tap_speaker_sentence</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>अब यह वाक्य पढ़िए — लड़की पौधों को पानी दे रही है। नीचे दो तस्वीरें हैं। पहली तस्वीर में लड़की फूल तोड़ रही है, और दूसरी तस्वीर में लड़की पौधों को पानी दे रही है। वाक्य के लिए सही तस्वीर दूसरी है, क्योंकि उसमें लड़की पौधों को पानी दे रही है।</t>
+          <t>वाक्य सुनने के लिए यहाँ टैप करिए।</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_cat_ok</t>
+          <t>vo_sent_boy_sit</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>बिल्ली दूध पी रही है।</t>
+          <t>लड़का पेड़ के नीचे बैठा है।</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_bird_ok</t>
+          <t>vo_t1_explain</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>चिड़िया पेड़ पर बैठी है।</t>
+          <t>चित्र में लड़का पेड़ के नीचे बैठा है। वाक्य में भी यही कहा गया है। इसलिए यह सही वाक्य है।</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_children_ok</t>
+          <t>vo_t2_instr</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>बच्चे मैदान में दौड़ रहे हैं।</t>
+          <t>ध्यान से देखिए। क्या यह वाक्य चित्र के लिए सही है?</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_cat_drink</t>
+          <t>vo_sent_girl_cycle</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए — किस तस्वीर में बिल्ली दूध पी रही है? उस तस्वीर पर टैप कीजिए।</t>
+          <t>लड़की साइकिल चला रही है।</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_boy_drink_ok</t>
+          <t>vo_t2_explain</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>लड़का पानी पी रहा है।</t>
+          <t>हाँ! यह वाक्य सही है। चित्र में लड़की साइकिल चला रही है और वाक्य में भी यही कहा गया है।</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_boy_sit</t>
+          <t>vo_t3_instr</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>लड़का पेड़ के नीचे बैठा है।</t>
+          <t>इस वाक्य के लिए सही चित्र चुनिए।</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_girl_cycle</t>
+          <t>vo_sent_girl_water</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>लड़की साइकिल चला रही है।</t>
+          <t>लड़की पौधों को पानी दे रही है।</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_boy_drink</t>
+          <t>vo_t3_explain</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए — तस्वीर में लड़का क्या कर रहा है? वह पानी पी रहा है। सही वाक्य पर टैप कीजिए।</t>
+          <t>इस वाक्य के लिए यह चित्र सही है।</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_mom_ok</t>
+          <t>vo_prompt_sent_to_pic</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>माँ अखबार पढ़ रही है।</t>
+          <t>वाक्य पढ़िए और सही चित्र चुनिए।</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_girl_read</t>
+          <t>vo_sent_cat_ok</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>लड़की किताब पढ़ रही है।</t>
+          <t>बिल्ली दूध पी रही है।</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_mom_water</t>
+          <t>vo_ok_pic</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>माँ पौधों को पानी दे रही है।</t>
+          <t>शाबाश! आपने सही चित्र चुना।</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_mom</t>
+          <t>vo_hint_cat_drink</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए — किस तस्वीर में माँ अखबार पढ़ रही है? उस तस्वीर पर टैप कीजिए।</t>
+          <t>ध्यान से देखिए और वह चित्र चुनिए जिसमें बिल्ली दूध पी रही है।</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_children_sit_ok</t>
+          <t>vo_prompt_pic_to_sent</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>बच्चे मैदान में बैठे हैं।</t>
+          <t>इस चित्र के लिए सही वाक्य चुनिए।</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_children</t>
+          <t>vo_sent_boy_drink_ok</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए — तस्वीर में बच्चे दौड़ रहे हैं या बैठे हैं?</t>
+          <t>लड़का पानी पी रहा है।</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_boy_fill_ok</t>
+          <t>vo_ok_sent_boy_drink</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>लड़का पानी भर रहा है।</t>
+          <t>शाबाश! आपने सही वाक्य चुना—लड़का पानी पी रहा है।</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_boy_eat</t>
+          <t>vo_sent_mom_ok</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>लड़का खाना खा रहा है।</t>
+          <t>माँ अखबार पढ़ रही है।</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_boy_fill</t>
+          <t>vo_hint_mom</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए — किस तस्वीर में लड़का पानी भर रहा है? उस तस्वीर पर टैप कीजिए।</t>
+          <t>ध्यान से देखिए और वह चित्र चुनिए जिसमें माँ अखबार पढ़ रही है।</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_goat_drink</t>
+          <t>vo_sent_children_sit_ok</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>बकरी पानी पी रही है।</t>
+          <t>बच्चे मैदान में बैठे हैं।</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_goat_ok</t>
+          <t>vo_sent_children_ok</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>बकरी घास खा रही है।</t>
+          <t>बच्चे मैदान में दौड़ रहे हैं।</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_goat_sit</t>
+          <t>vo_ok_sent_children_sit</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>बकरी घास पर बैठी है।</t>
+          <t>शाबाश! आपने सही वाक्य चुना—बच्चे मैदान में बैठे हैं।</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_goat</t>
+          <t>vo_sent_boy_fill_ok</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए — तस्वीर में बकरी क्या कर रही है? वह घास खा रही है। सही वाक्य पर टैप कीजिए।</t>
+          <t>लड़का पानी भर रहा है।</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_cat_sleep_ok</t>
+          <t>vo_hint_boy_fill</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>बिल्ली सो रही है।</t>
+          <t>ध्यान से देखिए और वह चित्र चुनिए जिसमें लड़का पानी भर रहा है।</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_cat_eat</t>
+          <t>vo_sent_goat_drink</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>बिल्ली खाना खा रही है।</t>
+          <t>बकरी पानी पी रही है।</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_cat</t>
+          <t>vo_sent_goat_ok</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए — किस तस्वीर में बिल्ली सो रही है? उस तस्वीर पर टैप कीजिए।</t>
+          <t>बकरी घास खा रही है।</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_bird_wrong</t>
+          <t>vo_sent_goat_sit</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>चिड़िया उड़ रही है।</t>
+          <t>बकरी घास पर बैठी है।</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_bird_peck_ok</t>
+          <t>vo_sent_cat_sleep_ok</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>चिड़िया दाना चुग रही है।</t>
+          <t>बिल्ली सो रही है।</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_bird_peck</t>
+          <t>vo_hint_cat</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए — तस्वीर में चिड़िया क्या कर रही है? वह दाना चुग रही है। सही वाक्य पर टैप कीजिए।</t>
+          <t>ध्यान से देखिए और वह चित्र चुनिए जिसमें बिल्ली सो रही है।</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>vo_prompt_pic_to_sent</t>
+          <t>vo_sent_bird_ok</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>इस तस्वीर के लिए सही वाक्य चुनिए।</t>
+          <t>चिड़िया पेड़ पर बैठी है।</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>vo_try_again</t>
+          <t>vo_sent_bird_wrong</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>फिर से कोशिश कीजिए।</t>
+          <t>चिड़िया उड़ रही है।</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>vo_reveal</t>
+          <t>vo_sent_bird_peck_ok</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>यह सही जोड़ा है।</t>
+          <t>चिड़िया दाना चुग रही है।</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>vo_well_done</t>
+          <t>vo_p5_instr</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>शाबाश! आपने तस्वीर और वाक्य का सही जोड़ा बनाना सीख लिया।</t>
+          <t>चलिए, एक खेल खेलते हैं। हर वाक्य को सही चित्र से मिलाइए।</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>vo_pt_tutorial</t>
+          <t>vo_p6_instr</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए और मेरे साथ जानिए। चलिए, शुरू करें!</t>
+          <t>अब चित्रों की बारी! हर चित्र को सही वाक्य से मिलाइए।</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>vo_pt_guided</t>
+          <t>vo_sent_grandpa_newspaper</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>बहुत बढ़िया! अब हम साथ मिलकर शुरू करते हैं। चलिए, साथ में करें!</t>
+          <t>दादाजी अखबार पढ़ रहे हैं।</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t>vo_sent_children_kite</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>बच्चे पतंग उड़ा रहे हैं।</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>vo_sent_dog_ball</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>कुत्ता गेंद से खेल रहा है।</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>vo_well_done</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>शाबाश! आपने चित्रों और वाक्यों को मिलाना सीख लिया!</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>vo_try_again</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>फिर से कोशिश कीजिए।</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>vo_reveal</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>यह सही जोड़ा है।</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>vo_pt_tutorial</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>ध्यान से देखिए और मेरे साथ जानिए। चलिए, शुरू करें!</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>vo_pt_guided</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>बहुत बढ़िया! अब हम साथ मिलकर शुरू करते हैं। चलिए, साथ में करें!</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>vo_pt_practice</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>वाह! अब आपकी बारी।</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B39"/>
+  <autoFilter ref="A1:B46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor code structure for improved readability and maintainability
</commit_message>
<xml_diff>
--- a/HI02H04_L01_S01/VO_Manifest.xlsx
+++ b/HI02H04_L01_S01/VO_Manifest.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VO Manifest" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'VO Manifest'!$A$1:$B$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'VO Manifest'!$A$1:$B$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -669,180 +669,180 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_boy_drink_ok</t>
+          <t>vo_sent_bird_ok</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>लड़का पानी पी रहा है।</t>
+          <t>चिड़िया पेड़ पर बैठी है।</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>vo_ok_sent_boy_drink</t>
+          <t>vo_sent_boy_drink_ok</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>शाबाश! आपने सही वाक्य चुना—लड़का पानी पी रहा है।</t>
+          <t>लड़का पानी पी रहा है।</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_mom_ok</t>
+          <t>vo_sent_goat_ok</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>माँ अखबार पढ़ रही है।</t>
+          <t>बकरी घास खा रही है।</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_mom</t>
+          <t>vo_ok_sent_boy_drink</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए और वह चित्र चुनिए जिसमें माँ अखबार पढ़ रही है।</t>
+          <t>शाबाश! आपने सही वाक्य चुना—लड़का पानी पी रहा है।</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_children_sit_ok</t>
+          <t>vo_sent_mom_ok</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>बच्चे मैदान में बैठे हैं।</t>
+          <t>माँ अखबार पढ़ रही है।</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_children_ok</t>
+          <t>vo_hint_mom</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>बच्चे मैदान में दौड़ रहे हैं।</t>
+          <t>ध्यान से देखिए और वह चित्र चुनिए जिसमें माँ अखबार पढ़ रही है।</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>vo_ok_sent_children_sit</t>
+          <t>vo_sent_children_sit_ok</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>शाबाश! आपने सही वाक्य चुना—बच्चे मैदान में बैठे हैं।</t>
+          <t>बच्चे मैदान में बैठे हैं।</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_boy_fill_ok</t>
+          <t>vo_sent_children_ok</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>लड़का पानी भर रहा है।</t>
+          <t>बच्चे मैदान में दौड़ रहे हैं।</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_boy_fill</t>
+          <t>vo_ok_sent_children_sit</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए और वह चित्र चुनिए जिसमें लड़का पानी भर रहा है।</t>
+          <t>शाबाश! आपने सही वाक्य चुना—बच्चे मैदान में बैठे हैं।</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_goat_drink</t>
+          <t>vo_sent_boy_fill_ok</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>बकरी पानी पी रही है।</t>
+          <t>लड़का पानी भर रहा है।</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_goat_ok</t>
+          <t>vo_hint_boy_fill</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>बकरी घास खा रही है।</t>
+          <t>ध्यान से देखिए और वह चित्र चुनिए जिसमें लड़का पानी भर रहा है।</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_goat_sit</t>
+          <t>vo_sent_goat_drink</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>बकरी घास पर बैठी है।</t>
+          <t>बकरी पानी पी रही है।</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_cat_sleep_ok</t>
+          <t>vo_sent_goat_sit</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>बिल्ली सो रही है।</t>
+          <t>बकरी घास पर बैठी है।</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>vo_hint_cat</t>
+          <t>vo_sent_cat_sleep_ok</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>ध्यान से देखिए और वह चित्र चुनिए जिसमें बिल्ली सो रही है।</t>
+          <t>बिल्ली सो रही है।</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>vo_sent_bird_ok</t>
+          <t>vo_hint_cat</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>चिड़िया पेड़ पर बैठी है।</t>
+          <t>ध्यान से देखिए और वह चित्र चुनिए जिसमें बिल्ली सो रही है।</t>
         </is>
       </c>
     </row>
@@ -942,68 +942,8 @@
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>vo_try_again</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>फिर से कोशिश कीजिए।</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>vo_reveal</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>यह सही जोड़ा है।</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>vo_pt_tutorial</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>ध्यान से देखिए और मेरे साथ जानिए। चलिए, शुरू करें!</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>vo_pt_guided</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>बहुत बढ़िया! अब हम साथ मिलकर शुरू करते हैं। चलिए, साथ में करें!</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>vo_pt_practice</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>वाह! अब आपकी बारी।</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B46"/>
+  <autoFilter ref="A1:B41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>